<commit_message>
Move YOLO workflow into HP60C startup workbook
</commit_message>
<xml_diff>
--- a/HP60C_网页抓取启动流程.xlsx
+++ b/HP60C_网页抓取启动流程.xlsx
@@ -13,6 +13,7 @@
     <sheet name="日志数据" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="故障排查" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="文件版本" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="YOLO on Orin" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总流程'!$A$1:$F$10</definedName>
@@ -21,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'日志数据'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'故障排查'!$A$1:$C$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'文件版本'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'YOLO on Orin'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1689,4 +1691,270 @@
   <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Command / Setting</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>When to Use</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Success Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="74" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Check Jetson Docker runtime</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>sudo docker run --rm --runtime nvidia nvcr.io/nvidia/l4t-base:35.4.1 bash -lc "ls /dev/nvhost* | head"</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run once after Docker/NVIDIA runtime setup</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Container prints /dev/nvhost-as-gpu and other /dev/nvhost* devices</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="74" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Create YOLO output directory</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>mkdir -p ~/hive_robot/DM_Control_Python/yolo_runs</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Before running YOLO predictions</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Directory exists on the Orin host</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="74" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Start YOLO JetPack 5 container</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>sudo docker run -it --rm \
+  --runtime nvidia \
+  --network host \
+  --ipc host \
+  -v ~/hive_robot:/workspace/hive_robot \
+  ultralytics/ultralytics:latest-jetson-jetpack5</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Use this on Orin JetPack 5 / L4T R35.x</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Shell prompt changes to root@ubuntu:/ultralytics#</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="74" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Verify CUDA and model loading</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>python3 - &lt;&lt;'PY'
+import torch
+from ultralytics import YOLO
+print('torch:', torch.__version__)
+print('cuda:', torch.cuda.is_available())
+if torch.cuda.is_available():
+    print('gpu:', torch.cuda.get_device_name(0))
+model = YOLO('yolo11n.pt')
+print('YOLO loaded')
+PY</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Inside the YOLO container</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Shows cuda: True, gpu: Orin, YOLO loaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="74" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Test built-in COCO image</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>yolo predict model=yolo11n.pt source=/ultralytics/ultralytics/assets/bus.jpg imgsz=640 conf=0.25</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Use this to confirm YOLO itself works</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Detects 4 persons and 1 bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="74" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Capture current HP60C frame</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ts=$(date +%s%3N)
+img=/tmp/hp60c_${ts}.jpg
+wget -O "$img" "http://127.0.0.1:8090/debug.jpg?t=${ts}"</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Use timestamp to avoid cached debug.jpg</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Creates a fresh /tmp/hp60c_&lt;timestamp&gt;.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="74" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Detect bottle and scissors on HP60C frame</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>yolo predict model=yolo11n.pt \
+  source="$img" \
+  imgsz=1280 \
+  conf=0.01 \
+  classes=39,76 \
+  project=/workspace/hive_robot/DM_Control_Python/yolo_runs \
+  name=bottle_scissors_${ts}</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Inside the YOLO container after capturing current HP60C frame</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Results saved under DM_Control_Python/yolo_runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Useful COCO class ids</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>bottle=39
+cell phone=67
+book=73
+scissors=76</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Use with classes=... to reduce noisy detections</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Class-limited detection is cleaner than all-class low-conf detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Testing note</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Default yolo11n.pt is only a COCO sanity check. HP60C overhead worktable images need class whitelist/per-class thresholds, then a custom HP60C chess/screw/object model.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Use when moving from demo detection to robot control</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Scissors detected reliably around 0.41-0.44; bottle was weak around 0.03 in testing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Log and sync left arm web control tuning
</commit_message>
<xml_diff>
--- a/HP60C_网页抓取启动流程.xlsx
+++ b/HP60C_网页抓取启动流程.xlsx
@@ -8,21 +8,22 @@
   </bookViews>
   <sheets>
     <sheet name="总流程" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="命令速查" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="网页按钮" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="日志数据" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="故障排查" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="文件版本" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="YOLO on Orin" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="左臂v2.5.3启动" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="命令速查" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="网页按钮" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="日志数据" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="故障排查" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="文件版本" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="YOLO on Orin" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总流程'!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'命令速查'!$A$1:$C$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'网页按钮'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'日志数据'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'故障排查'!$A$1:$C$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'文件版本'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'YOLO on Orin'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'命令速查'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'网页按钮'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'日志数据'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'故障排查'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'文件版本'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'YOLO on Orin'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,10 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -72,7 +77,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -94,11 +99,25 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -110,6 +129,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -477,317 +502,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>步骤</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>位置</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>命令 / 操作</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>注意事项</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>成功标志</t>
         </is>
       </c>
     </row>
     <row r="2" ht="78" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Orin 开机并登录</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Orin</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>开机后登录 nvidia 用户，确认 HP60C、机械臂 CAN/电源已连接。</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>只做硬件准备</t>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>开机后登录 nvidia 用户，确认 HP60C、左臂 CAN、机械臂电源已连接。</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>不要先执行机械臂动作。</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>硬件准备完成</t>
         </is>
       </c>
     </row>
     <row r="3" ht="78" customHeight="1">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>启动 HP60C ROS 驱动</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Orin 终端 1</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>cd ~/ascam_ws
 source ~/.bashrc
 roslaunch ascamera hp60c.launch</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>保持终端不关闭</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>正常会启动 ROS master 和相机 topic</t>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>保持终端不关闭。这个窗口负责相机 ROS topic。</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>看到相机节点启动，无报错退出</t>
         </is>
       </c>
     </row>
     <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>首次配置免密 sudo（只需一次）</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>首次配置 left_arm_v2_5_3.py 免密 sudo</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Orin 终端 2</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>cd ~/hive_robot/DM_Control_Python
-sudo bash install_hive_robot_sudoers.sh /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py
-sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py status</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>只允许 left_arm_controller.py 免密，不是全局免密</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>第二条 status 不要求密码即成功</t>
+sudo bash install_hive_robot_sudoers.sh /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py
+sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py status</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>只需一次；如果 web 输出 sudo password required，重新做这一步。</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>status 不要求密码且能读到电机状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>启动网页推流和控制服务</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>启动 v2.5.3 web 控制平台</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Orin 终端 2</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>cd ~/hive_robot/DM_Control_Python
-python3 hp60c_stream_server.py --scan-windows --window-w 80 --window-h 85 --window-step 20 --min-area 30 --max-area 6000 --aim-y-frac 0.25 --target-depth-percentile 75 --port 8090 --enable-controller-execute</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>服务启动后不要关闭该终端</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>看到 Controller execute enabled: True</t>
+python3 left_arm_v2_5_3_web_control.py --enable-execute --port 8091</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>保持终端不关闭。默认会启用 RGB-D 流、绿色 ROI、XYZ、按钮控制。</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>看到 Web controller version: v1.2 和 listening on 0.0.0.0:8091</t>
         </is>
       </c>
     </row>
     <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Windows 打开网页</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Windows 浏览器</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>http://&lt;orin-ip&gt;:8090/</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>如果不知道 IP，在 Orin 上用 hostname -I 查看</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>能看到实时画面、紫框、黄圈</t>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>http://&lt;orin-ip&gt;:8091/</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>如果不知道 IP，在 Orin 上运行 hostname -I。</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>能看到 RGB-D 画面、绿色 ROI、Forward/Left/Up/Depth</t>
         </is>
       </c>
     </row>
     <row r="7" ht="78" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>先验证姿态</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>确认视频流和 XYZ</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Windows 网页</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>勾选 skip claw -&gt; 点击 执行当前目标</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>机械臂会运动，但不会闭爪</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>确认侧摆、手肘、手腕姿态正确</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>观察 /stream.mjpg；右侧 Status 查看 Forward、Left、Up、Depth。</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>如果无画面，先确认终端 1 的 roslaunch 还在运行。</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>绿色框和 XYZ 数据正常刷新</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>正式抓取</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Capture / Move</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Windows 网页</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>取消 skip claw -&gt; 点击 执行当前目标</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>机械臂会闭爪抓取</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>观察是否抓到目标物</t>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Capture New Home
+Capture New Clearance
+Table Clearance Move
+Home Move</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Capture 会覆盖 data 里的 home/clearance pose；执行前确认机械臂已在目标姿态。</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Debug Output 返回 returncode=0</t>
         </is>
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>记录结果</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>独立关节微调 v1.2</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Windows 网页</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>点击 记录完美 / 记录成功 / 记录失败，并输入备注</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>失败备注写清楚：手腕/侧摆/肘/前摆怎么偏</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>记录写入 data/hp60c_web_runs.jsonl</t>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>在 Joint Nudge 选择 2° / 5° / 10°，点击对应关节方向按钮。</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>优先小角度；elbow 接近物理极限，不建议在 clearance 后 nudge。</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>nudge-hold 输出 returncode=0，关节无抖动</t>
         </is>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>回 Home</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Debug Output 复制</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Windows 网页</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>点击 Home</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>执行 sudo -n python3 left_arm_controller.py home</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>机械臂安全回 home</t>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>点击 Debug Output 右上角 Copy。</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>用于把完整 stdout/stderr 发给 Codex 分析。</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Status 显示 Debug output copied</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Emergency Stop / 关机</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Windows 网页 / Orin</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>网页点击 Emergency Stop
+或终端 sudo poweroff</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>关机前确认没有机械臂动作在运行。</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>电机禁用或系统关机</t>
         </is>
       </c>
     </row>
@@ -803,202 +866,742 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>模块</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>当前值 / 命令</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>版本</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>web controller</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3_web_control.py v1.2</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>新增 Joint Nudge、Copy、ROI、XYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>端口</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>网页地址</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>http://&lt;orin-ip&gt;:8091/</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>旧抓取 server 默认 8090，新左臂控制平台默认 8091</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>终端 1</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>相机 ROS</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>cd ~/ascam_ws
+source ~/.bashrc
+roslaunch ascamera hp60c.launch</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>必须保持运行</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>终端 2</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>web controller</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>cd ~/hive_robot/DM_Control_Python
+python3 left_arm_v2_5_3_web_control.py --enable-execute --port 8091</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>必须保持运行</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>视频流</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>RGB + Depth</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>/stream.mjpg</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>网页首页默认使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>视频流</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>RGB only</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>/rgb.mjpg</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>调 RGB 时用</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>视频流</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Depth only</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>/depth.mjpg</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>调 depth 时用</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>绿色框默认值</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>x0=55, y0=115, x1=605, y1=455</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>可用 --roi-x0/y0/x1/y1 覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>相机物理模型</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>forward=10.5cm, left=-13.0cm, up=12.0cm, pitch_down=70°</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>参考点是 shoulder_front 轴心</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>按钮</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Capture New Home</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3.py capture-home --note web-control</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>覆盖 home pose</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>按钮</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Capture New Clearance</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3.py capture-clearance --note web-control</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>覆盖 table clearance pose</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>按钮</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Table Clearance Move</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3.py clearance --deadband-deg 0.5 --max-delta-deg 120 --step-deg 5 --execute</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>10s 六联动稳定版</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>按钮</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Home Move</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3.py home --deadband-deg 0.5 --max-delta-deg 120 --execute</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>16s 六联动 home</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>按钮</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Emergency Stop</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>disable DEFAULT_JOINTS</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>会先尝试停止当前 web 启动的进程</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Joint Nudge</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>度数</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>2° / 5° / 10°</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>每次弹确认，同一时刻只允许一个动作</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Joint Nudge</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>执行方式</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3.py nudge-hold --hold-joints shoulder_front,shoulder_side,shoulder_rotate,elbow,arm_roll,wrist_side,wrist --auto-gains</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>主动关节移动，其它 6 个关节 hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Joint Nudge</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>wrist 稳定参数</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>kp=26.0, kd=4.7, seconds=6.0</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>复用 clearance wrist fine 参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Joint Nudge</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>shoulder_front 防下坠</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>hold_tau shoulder_front=2.5</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>nudge-hold 会传 CLEARANCE_JOINT_HOLD_TAU</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Debug</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Copy</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Debug Output 右上角 Copy</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>HTTP 环境下使用 clipboard fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>日志</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>web run log</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>/home/nvidia/hive_robot/DM_Control_Python/data/left_arm_v2_5_3_web_runs.jsonl</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>记录 button/nudge stdout/stderr</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>用途</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>命令</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>什么时候用</t>
         </is>
       </c>
     </row>
     <row r="2" ht="70" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>启动 HP60C ROS</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>cd ~/ascam_ws
 source ~/.bashrc
 roslaunch ascamera hp60c.launch</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>每次开机后先运行，保持终端打开</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>查看 Orin IP</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>hostname -I</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Windows 浏览器需要 http://&lt;orin-ip&gt;:8090/</t>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Windows 浏览器需要 http://&lt;orin-ip&gt;:8091/</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>安装免密 sudo</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>安装 v2.5.3 免密 sudo</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>cd ~/hive_robot/DM_Control_Python
-sudo bash install_hive_robot_sudoers.sh /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+sudo bash install_hive_robot_sudoers.sh /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>只需一次；换路径/重装系统后再做</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>测试免密 sudo</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py status</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>测试 v2.5.3 免密 sudo</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py status</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>不提示密码即成功</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>启动网页控制服务</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>启动新 web 控制平台</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>cd ~/hive_robot/DM_Control_Python
-python3 hp60c_stream_server.py --scan-windows --window-w 80 --window-h 85 --window-step 20 --min-area 30 --max-area 6000 --aim-y-frac 0.25 --target-depth-percentile 75 --port 8090 --enable-controller-execute</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>每次测试抓取前运行</t>
+python3 left_arm_v2_5_3_web_control.py --enable-execute --port 8091</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>当前推荐流程；含 RGB-D、绿色 ROI、XYZ、home/clearance、nudge-hold</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>只看流，不允许网页控制</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>python3 hp60c_stream_server.py --scan-windows --window-w 80 --window-h 85 --window-step 20 --min-area 30 --max-area 6000 --aim-y-frac 0.25 --target-depth-percentile 75 --port 8090</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>调相机/看画面时用</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>只看流，不允许网页执行</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>cd ~/hive_robot/DM_Control_Python
+python3 left_arm_v2_5_3_web_control.py --port 8091</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>调视频/看 XYZ 时用，不允许按钮执行机械臂动作</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>手动执行当前命令</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py target-shoulder --forward &lt;F&gt; --left &lt;L&gt; --up &lt;U&gt; --geometry-execution-blend 1.00 --execute --allow-unverified-geometry</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>网页复制命令后可粘贴到终端</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>自定义 ROI 启动</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>python3 left_arm_v2_5_3_web_control.py --enable-execute --port 8091 --roi-x0 55 --roi-y0 115 --roi-x1 605 --roi-y1 455</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>绿色框需要调整时用</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>手动回 Home</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_controller.py home</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>当前相机物理参数</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>--camera-forward-from-shoulder-cm 10.5
+--camera-left-from-shoulder-cm -13.0
+--camera-up-from-shoulder-cm 12.0
+--camera-pitch-down-deg 70.0</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>默认已写入脚本；只有重新标定时才需要覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>手动 Table Clearance</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py clearance --deadband-deg 0.5 --max-delta-deg 120 --step-deg 5 --execute</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>网页按钮无响应时备用</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>手动 Home</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py home --deadband-deg 0.5 --max-delta-deg 120 --execute</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>网页 Home 无响应时备用</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>查看最近训练日志</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>tail -n 20 /home/nvidia/hive_robot/DM_Control_Python/data/hp60c_web_runs.jsonl</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>把最近记录发给 Codex 分析</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>备份训练日志</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>cp /home/nvidia/hive_robot/DM_Control_Python/data/hp60c_web_runs.jsonl ~/hp60c_web_runs_$(date +%Y%m%d_%H%M%S).jsonl</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>一天测试结束后备份</t>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>查看 clearance pose</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py show-clearance</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>对比 table clearance 位置数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>wrist forward 5° nudge-hold</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>sudo -n python3 /home/nvidia/hive_robot/DM_Control_Python/left_arm_v2_5_3.py nudge-hold --joint wrist --deg 5 --seconds 6 --max-deg 10 --hold-joints shoulder_front,shoulder_side,shoulder_rotate,elbow,arm_roll,wrist_side,wrist --auto-gains</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>clearance holding 后单独微调 wrist，防抖版本</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>查看 web 运行日志</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>tail -n 30 /home/nvidia/hive_robot/DM_Control_Python/data/left_arm_v2_5_3_web_runs.jsonl</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>把最近执行记录发给 Codex 分析</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1227,7 +1830,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1383,7 +1986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1590,13 +2193,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1604,86 +2207,98 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>字段</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>生成日期</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>更新日期</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>适用目录</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>~/hive_robot/DM_Control_Python</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>主要脚本</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>hp60c_stream_server.py, left_arm_controller.py, install_hive_robot_sudoers.sh</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>新主要脚本</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>left_arm_v2_5_3_web_control.py, left_arm_v2_5_3.py, install_hive_robot_sudoers.sh</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>网页地址</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>http://&lt;orin-ip&gt;:8090/</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>新网页地址</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>http://&lt;orin-ip&gt;:8091/</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>控制模式</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>target-shoulder, geometry-execution-blend=1.00</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>新控制模式</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>home/clearance/nudge-hold web controller v1.2</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>默认日志</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>data/hp60c_web_runs.jsonl</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>新默认日志</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>data/left_arm_v2_5_3_web_runs.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>旧版抓取脚本</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>hp60c_stream_server.py, left_arm_controller.py 仍保留在其它 sheet 作为历史参考</t>
         </is>
       </c>
     </row>
@@ -1693,7 +2308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>